<commit_message>
Plantilla Flujo de Caja: categorías de empresa en lugar de personales
Ingresos: ventas de contado, cobro de cartera, anticipos de clientes, etc.
Egresos: proveedores, nómina, seguridad social, impuestos, arriendo, etc.
Se conservan fórmulas, tablas, gráficos y validaciones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MUKfhfeK5agqgnqEvVQUqQ
</commit_message>
<xml_diff>
--- a/Plantillas/Fp_Flujo_de_caja_mensual.xlsx
+++ b/Plantillas/Fp_Flujo_de_caja_mensual.xlsx
@@ -22,7 +22,7 @@
     <definedName name="Mes">Dashboard!$E$6</definedName>
     <definedName name="SaldoInicial">Configuración!$E$8</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -66,19 +66,19 @@
     <t>Categorías de Ingresos</t>
   </si>
   <si>
-    <t>Sueldo</t>
+    <t>Ventas de contado</t>
   </si>
   <si>
-    <t>Bonos</t>
+    <t>Cobro de cartera</t>
   </si>
   <si>
-    <t>Freelance</t>
+    <t>Anticipos de clientes</t>
   </si>
   <si>
-    <t>Inversiones</t>
+    <t>Rendimientos financieros</t>
   </si>
   <si>
-    <t>Reembolsos</t>
+    <t>Préstamos recibidos</t>
   </si>
   <si>
     <t>Otros ingresos</t>
@@ -87,37 +87,37 @@
     <t>Categorías de Egresos</t>
   </si>
   <si>
-    <t>Comida</t>
+    <t>Proveedores</t>
   </si>
   <si>
-    <t>Transporte</t>
+    <t>Transporte y fletes</t>
   </si>
   <si>
-    <t>Vivienda/Alquiler</t>
+    <t>Arriendo</t>
   </si>
   <si>
-    <t>Servicios (luz, agua, gas)</t>
+    <t>Servicios públicos</t>
   </si>
   <si>
-    <t>Internet/Teléfono</t>
+    <t>Internet y telefonía</t>
   </si>
   <si>
-    <t>Salud</t>
+    <t>Seguridad social</t>
   </si>
   <si>
-    <t>Educación</t>
+    <t>Nómina</t>
   </si>
   <si>
-    <t>Ocio/Entretenimiento</t>
+    <t>Impuestos</t>
   </si>
   <si>
-    <t>Ropa</t>
+    <t>Publicidad y mercadeo</t>
   </si>
   <si>
-    <t>Ahorro/Inversión</t>
+    <t>Compra de equipos</t>
   </si>
   <si>
-    <t>Deudas/Préstamos</t>
+    <t>Pago de créditos</t>
   </si>
   <si>
     <t>Otros gastos</t>
@@ -165,13 +165,13 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Sueldo mensual</t>
+    <t>Venta de contado del día</t>
   </si>
   <si>
-    <t>Supermercado semanal</t>
+    <t>Pago a proveedor de insumos</t>
   </si>
   <si>
-    <t>Carga de combustible</t>
+    <t>Flete de despacho</t>
   </si>
   <si>
     <t>info@DataEdgeConsulting.onmicrosoft.com</t>
@@ -246,7 +246,7 @@
     <t>TOP 5 CATEGORÍAS DE GASTO (MES ACTUAL)</t>
   </si>
   <si>
-    <t>Extra</t>
+    <t>Ingreso no operacional</t>
   </si>
 </sst>
 </file>
@@ -1576,10 +1576,10 @@
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Comida</c:v>
+                  <c:v>Proveedores</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Transporte</c:v>
+                  <c:v>Transporte y fletes</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6814,7 +6814,7 @@
       </c>
       <c r="J8" s="71" t="str">
         <f>IF(IFERROR(LARGE($N$8:$N$19,1),-1)&lt;=0,"",IFERROR(INDEX($M$8:$M$19,MATCH(LARGE($N$8:$N$19,1),$N$8:$N$19,0)),""))</f>
-        <v>Comida</v>
+        <v>Proveedores</v>
       </c>
       <c r="K8" s="68">
         <f>IFERROR(IF(LARGE($N$8:$N$19,1)&lt;=0,0,ROUND(LARGE($N$8:$N$19,1),2)),0)</f>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="M8" t="str">
         <f>Configuración!F12</f>
-        <v>Comida</v>
+        <v>Proveedores</v>
       </c>
       <c r="N8">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M8,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="J9" s="72" t="str">
         <f>IF(IFERROR(LARGE($N$8:$N$19,2),-1)&lt;=0,"",IFERROR(INDEX($M$8:$M$19,MATCH(LARGE($N$8:$N$19,2),$N$8:$N$19,0)),""))</f>
-        <v>Transporte</v>
+        <v>Transporte y fletes</v>
       </c>
       <c r="K9" s="70">
         <f>IFERROR(IF(LARGE($N$8:$N$19,2)&lt;=0,0,ROUND(LARGE($N$8:$N$19,2),2)),0)</f>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="M9" t="str">
         <f>Configuración!F13</f>
-        <v>Transporte</v>
+        <v>Transporte y fletes</v>
       </c>
       <c r="N9">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M9,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -6888,7 +6888,7 @@
       </c>
       <c r="M10" t="str">
         <f>Configuración!F14</f>
-        <v>Vivienda/Alquiler</v>
+        <v>Arriendo</v>
       </c>
       <c r="N10">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M10,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="M11" t="str">
         <f>Configuración!F15</f>
-        <v>Servicios (luz, agua, gas)</v>
+        <v>Servicios públicos</v>
       </c>
       <c r="N11">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M11,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -6954,7 +6954,7 @@
       </c>
       <c r="M12" t="str">
         <f>Configuración!F16</f>
-        <v>Internet/Teléfono</v>
+        <v>Internet y telefonía</v>
       </c>
       <c r="N12">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M12,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -6976,7 +6976,7 @@
       </c>
       <c r="M13" t="str">
         <f>Configuración!F17</f>
-        <v>Salud</v>
+        <v>Seguridad social</v>
       </c>
       <c r="N13">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M13,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="M14" t="str">
         <f>Configuración!F18</f>
-        <v>Educación</v>
+        <v>Nómina</v>
       </c>
       <c r="N14">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M14,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="M15" t="str">
         <f>Configuración!F19</f>
-        <v>Ocio/Entretenimiento</v>
+        <v>Impuestos</v>
       </c>
       <c r="N15">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M15,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="M16" t="str">
         <f>Configuración!F20</f>
-        <v>Ropa</v>
+        <v>Publicidad y mercadeo</v>
       </c>
       <c r="N16">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M16,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="M17" t="str">
         <f>Configuración!F21</f>
-        <v>Ahorro/Inversión</v>
+        <v>Compra de equipos</v>
       </c>
       <c r="N17">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M17,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="M18" t="str">
         <f>Configuración!F22</f>
-        <v>Deudas/Préstamos</v>
+        <v>Pago de créditos</v>
       </c>
       <c r="N18">
         <f>SUMIFS(tblMov[Egreso],tblMov[Categoría],M18,tblMov[Fecha],"&gt;="&amp;DATE(Anio,Mes,1),tblMov[Fecha],"&lt;="&amp;EOMONTH(DATE(Anio,Mes,1),0))-ROW()/1000000</f>

</xml_diff>